<commit_message>
feat: tambah fitur CRUD, import, export detail dan retur penjualan
</commit_message>
<xml_diff>
--- a/PWLPOS/public/template_penjualan.xlsx
+++ b/PWLPOS/public/template_penjualan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\laragon\www\WebLanjut\PWLPOS\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1680801C-9288-4272-87BC-3118C1E9C6BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DBA6222-3281-49A2-AAD4-C806ACBB1FFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2535" yWindow="2820" windowWidth="8865" windowHeight="7995" xr2:uid="{E70CEA3A-F66A-4856-B43A-FFD0CFD883A8}"/>
+    <workbookView xWindow="390" yWindow="390" windowWidth="8865" windowHeight="7995" xr2:uid="{E70CEA3A-F66A-4856-B43A-FFD0CFD883A8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Budi Santoso</t>
   </si>
@@ -45,43 +45,25 @@
     <t>Tanggal Penjualan</t>
   </si>
   <si>
-    <t>Aldi Setiawan</t>
-  </si>
-  <si>
-    <t>PS123456</t>
-  </si>
-  <si>
-    <t>Rina Permata</t>
-  </si>
-  <si>
-    <t>Andi Pratama</t>
-  </si>
-  <si>
-    <t>PS123457</t>
-  </si>
-  <si>
     <t>Joko Widodo</t>
   </si>
   <si>
-    <t>Tina Sari</t>
-  </si>
-  <si>
-    <t>PS123458</t>
-  </si>
-  <si>
-    <t>Siti Aisyah</t>
-  </si>
-  <si>
-    <t>Fauzan Abdullah</t>
-  </si>
-  <si>
-    <t>PS123459</t>
-  </si>
-  <si>
-    <t>Mochammad Iqbal</t>
-  </si>
-  <si>
-    <t>PS123460</t>
+    <t>PNJ001</t>
+  </si>
+  <si>
+    <t>Siti Aminah</t>
+  </si>
+  <si>
+    <t>PNJ002</t>
+  </si>
+  <si>
+    <t>PNJ003</t>
+  </si>
+  <si>
+    <t>PNJ004</t>
+  </si>
+  <si>
+    <t>04/13/2025</t>
   </si>
 </sst>
 </file>
@@ -450,7 +432,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53275FDE-D7D2-4F79-A64F-121251CD8485}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.28515625" bestFit="1" customWidth="1"/>
@@ -474,8 +456,8 @@
       </c>
     </row>
     <row r="2" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>6</v>
+      <c r="A2" s="2">
+        <v>3</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>0</v>
@@ -484,63 +466,49 @@
         <v>7</v>
       </c>
       <c r="D2" s="3">
-        <v>45757</v>
+        <v>45934</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="2">
+        <v>3</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>10</v>
-      </c>
       <c r="D3" s="3">
-        <v>45758</v>
+        <v>45965</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>11</v>
+      <c r="A4" s="2">
+        <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D4" s="3">
-        <v>45759</v>
+        <v>45995</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>14</v>
+      <c r="A5" s="2">
+        <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D5" s="3">
-        <v>45760</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D6" s="3">
-        <v>45761</v>
+        <v>11</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>